<commit_message>
Size header rows from the longest heading so wrapped headers stop clipping
Excel does not auto-grow a row whose height you have set, so two-line headings
like the branch-summary columns lost their second line. header_row now derives
the height from the longest header measured against its own column width.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo/דוח-כספי-לדוגמה.xlsx
+++ b/demo/דוח-כספי-לדוגמה.xlsx
@@ -1302,7 +1302,7 @@
       <c r="H23" s="4" t="n"/>
       <c r="I23" s="4" t="n"/>
     </row>
-    <row r="24" ht="32" customHeight="1">
+    <row r="24" ht="48" customHeight="1">
       <c r="A24" s="13" t="inlineStr">
         <is>
           <t>חנות</t>
@@ -1700,7 +1700,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1">
+    <row r="4" ht="34" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
           <t>פרמטר</t>
@@ -1881,7 +1881,7 @@
       <c r="L13" s="4" t="n"/>
       <c r="M13" s="4" t="n"/>
     </row>
-    <row r="14" ht="32" customHeight="1">
+    <row r="14" ht="34" customHeight="1">
       <c r="A14" s="13" t="inlineStr">
         <is>
           <t>חודש</t>
@@ -2042,7 +2042,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1">
+    <row r="4" ht="48" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
           <t>מק״ט</t>
@@ -6423,7 +6423,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1">
+    <row r="4" ht="48" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
           <t>חנות</t>
@@ -6755,7 +6755,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1">
+    <row r="4" ht="34" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
           <t>חנות</t>
@@ -7284,7 +7284,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1">
+    <row r="4" ht="34" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
           <t>סעיף הוצאה</t>
@@ -7882,7 +7882,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1">
+    <row r="4" ht="34" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
           <t>סעיף</t>
@@ -8546,7 +8546,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="32" customHeight="1">
+    <row r="4" ht="34" customHeight="1">
       <c r="A4" s="13" t="inlineStr">
         <is>
           <t>חודש</t>

</xml_diff>